<commit_message>
Drive URL conversion, existing-ID reuse, multi-variant, browser_addon
- Drive sharing links (drive.google.com/file/d/<ID>, ?id=<ID>) are
  auto-rewritten to lh3.googleusercontent.com/d/<ID> so Meta's fetcher
  can actually load them.
- existing_campaign_id / existing_adset_id columns let new ad sets
  attach to an existing campaign, or new ads to an existing ad set,
  instead of always creating fresh.
- Pipe-separated values in primary_text / headline / description switch
  the creative to asset_feed_spec with multiple variants (image gets
  uploaded to /adimages first to obtain a hash, since asset_feed_spec
  only accepts hashes).
- display_link populates link_data.caption (or asset_feed_spec
  link_urls[].display_url).
- threads_user_id added to object_story_spec.
- browser_addon dropdown (NONE / CALL / MESSENGER / WHATSAPP) replaces
  the cta when set; CALL and WHATSAPP require phone_number.
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -413,370 +413,406 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AW2"/>
+  <dimension ref="A1:BC2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="23" customWidth="1" min="4" max="4"/>
-    <col width="27" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
-    <col width="23" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
-    <col width="21" customWidth="1" min="9" max="9"/>
-    <col width="20" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="18" customWidth="1" min="12" max="12"/>
-    <col width="21" customWidth="1" min="13" max="13"/>
-    <col width="14" customWidth="1" min="14" max="14"/>
-    <col width="16" customWidth="1" min="15" max="15"/>
-    <col width="16" customWidth="1" min="16" max="16"/>
-    <col width="21" customWidth="1" min="17" max="17"/>
-    <col width="24" customWidth="1" min="18" max="18"/>
-    <col width="14" customWidth="1" min="19" max="19"/>
-    <col width="15" customWidth="1" min="20" max="20"/>
-    <col width="19" customWidth="1" min="21" max="21"/>
-    <col width="18" customWidth="1" min="22" max="22"/>
-    <col width="14" customWidth="1" min="23" max="23"/>
-    <col width="14" customWidth="1" min="24" max="24"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="23" customWidth="1" min="5" max="5"/>
+    <col width="27" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="23" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="21" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="19" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="21" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="16" customWidth="1" min="17" max="17"/>
+    <col width="16" customWidth="1" min="18" max="18"/>
+    <col width="21" customWidth="1" min="19" max="19"/>
+    <col width="24" customWidth="1" min="20" max="20"/>
+    <col width="14" customWidth="1" min="21" max="21"/>
+    <col width="15" customWidth="1" min="22" max="22"/>
+    <col width="19" customWidth="1" min="23" max="23"/>
+    <col width="18" customWidth="1" min="24" max="24"/>
     <col width="14" customWidth="1" min="25" max="25"/>
-    <col width="19" customWidth="1" min="26" max="26"/>
-    <col width="16" customWidth="1" min="27" max="27"/>
-    <col width="18" customWidth="1" min="28" max="28"/>
-    <col width="17" customWidth="1" min="29" max="29"/>
-    <col width="14" customWidth="1" min="30" max="30"/>
-    <col width="19" customWidth="1" min="31" max="31"/>
+    <col width="14" customWidth="1" min="26" max="26"/>
+    <col width="14" customWidth="1" min="27" max="27"/>
+    <col width="19" customWidth="1" min="28" max="28"/>
+    <col width="16" customWidth="1" min="29" max="29"/>
+    <col width="18" customWidth="1" min="30" max="30"/>
+    <col width="17" customWidth="1" min="31" max="31"/>
     <col width="14" customWidth="1" min="32" max="32"/>
-    <col width="14" customWidth="1" min="33" max="33"/>
+    <col width="19" customWidth="1" min="33" max="33"/>
     <col width="14" customWidth="1" min="34" max="34"/>
     <col width="14" customWidth="1" min="35" max="35"/>
-    <col width="30" customWidth="1" min="36" max="36"/>
-    <col width="30" customWidth="1" min="37" max="37"/>
-    <col width="14" customWidth="1" min="38" max="38"/>
-    <col width="20" customWidth="1" min="39" max="39"/>
+    <col width="14" customWidth="1" min="36" max="36"/>
+    <col width="14" customWidth="1" min="37" max="37"/>
+    <col width="30" customWidth="1" min="38" max="38"/>
+    <col width="30" customWidth="1" min="39" max="39"/>
     <col width="14" customWidth="1" min="40" max="40"/>
-    <col width="14" customWidth="1" min="41" max="41"/>
-    <col width="14" customWidth="1" min="42" max="42"/>
+    <col width="20" customWidth="1" min="41" max="41"/>
+    <col width="17" customWidth="1" min="42" max="42"/>
     <col width="14" customWidth="1" min="43" max="43"/>
     <col width="14" customWidth="1" min="44" max="44"/>
     <col width="14" customWidth="1" min="45" max="45"/>
     <col width="14" customWidth="1" min="46" max="46"/>
     <col width="14" customWidth="1" min="47" max="47"/>
     <col width="14" customWidth="1" min="48" max="48"/>
-    <col width="19" customWidth="1" min="49" max="49"/>
+    <col width="14" customWidth="1" min="49" max="49"/>
+    <col width="14" customWidth="1" min="50" max="50"/>
+    <col width="14" customWidth="1" min="51" max="51"/>
+    <col width="14" customWidth="1" min="52" max="52"/>
+    <col width="15" customWidth="1" min="53" max="53"/>
+    <col width="14" customWidth="1" min="54" max="54"/>
+    <col width="19" customWidth="1" min="55" max="55"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>existing_campaign_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>campaign_name</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>campaign_objective</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>buying_type</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>special_ad_categories</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>campaign_daily_budget_usd</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>campaign_lifetime_budget_usd</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>campaign_bid_strategy</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>campaign_spend_cap_usd</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>campaign_start_time</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>campaign_stop_time</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>existing_adset_id</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
         <is>
           <t>adset_name</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>daily_budget_usd</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>lifetime_budget_usd</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>bid_strategy</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>bid_amount_usd</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>bid_roas_floor</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>daily_spend_cap_usd</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>lifetime_spend_cap_usd</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>pacing_type</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>billing_event</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>optimization_goal</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>destination_type</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>start_time</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>end_time</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>pixel_id</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>custom_event_type</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>application_id</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>object_store_url</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>dsa_beneficiary</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>dsa_payor</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>saved_audience_id</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>countries</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>age_min</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>age_max</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AK1" t="inlineStr">
         <is>
           <t>genders</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AL1" t="inlineStr">
         <is>
           <t>included_custom_audience_ids</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="AM1" t="inlineStr">
         <is>
           <t>excluded_custom_audience_ids</t>
         </is>
       </c>
-      <c r="AL1" t="inlineStr">
+      <c r="AN1" t="inlineStr">
         <is>
           <t>page_id</t>
         </is>
       </c>
-      <c r="AM1" t="inlineStr">
+      <c r="AO1" t="inlineStr">
         <is>
           <t>instagram_actor_id</t>
         </is>
       </c>
-      <c r="AN1" t="inlineStr">
+      <c r="AP1" t="inlineStr">
+        <is>
+          <t>threads_user_id</t>
+        </is>
+      </c>
+      <c r="AQ1" t="inlineStr">
         <is>
           <t>ad_name</t>
         </is>
       </c>
-      <c r="AO1" t="inlineStr">
+      <c r="AR1" t="inlineStr">
         <is>
           <t>image_url</t>
         </is>
       </c>
-      <c r="AP1" t="inlineStr">
+      <c r="AS1" t="inlineStr">
         <is>
           <t>video_id</t>
         </is>
       </c>
-      <c r="AQ1" t="inlineStr">
+      <c r="AT1" t="inlineStr">
         <is>
           <t>primary_text</t>
         </is>
       </c>
-      <c r="AR1" t="inlineStr">
+      <c r="AU1" t="inlineStr">
         <is>
           <t>headline</t>
         </is>
       </c>
-      <c r="AS1" t="inlineStr">
+      <c r="AV1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="AT1" t="inlineStr">
+      <c r="AW1" t="inlineStr">
         <is>
           <t>link_url</t>
         </is>
       </c>
-      <c r="AU1" t="inlineStr">
+      <c r="AX1" t="inlineStr">
+        <is>
+          <t>display_link</t>
+        </is>
+      </c>
+      <c r="AY1" t="inlineStr">
         <is>
           <t>url_tags</t>
         </is>
       </c>
-      <c r="AV1" t="inlineStr">
+      <c r="AZ1" t="inlineStr">
         <is>
           <t>cta</t>
         </is>
       </c>
-      <c r="AW1" t="inlineStr">
+      <c r="BA1" t="inlineStr">
+        <is>
+          <t>browser_addon</t>
+        </is>
+      </c>
+      <c r="BB1" t="inlineStr">
+        <is>
+          <t>phone_number</t>
+        </is>
+      </c>
+      <c r="BC1" t="inlineStr">
         <is>
           <t>conversion_domain</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" t="inlineStr"/>
+      <c r="B2" t="inlineStr">
         <is>
           <t>Spring Launch</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>OUTCOME_TRAFFIC</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>AUCTION</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>NONE</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
         <is>
           <t>US Broad 25-54</t>
         </is>
       </c>
-      <c r="L2" t="n">
+      <c r="N2" t="n">
         <v>50</v>
       </c>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr">
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr">
         <is>
           <t>LOWEST_COST_WITHOUT_CAP</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr"/>
-      <c r="T2" t="inlineStr">
+      <c r="T2" t="inlineStr"/>
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr">
         <is>
           <t>IMPRESSIONS</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
+      <c r="W2" t="inlineStr">
         <is>
           <t>LANDING_PAGE_VIEWS</t>
         </is>
       </c>
-      <c r="V2" t="inlineStr">
+      <c r="X2" t="inlineStr">
         <is>
           <t>WEBSITE</t>
         </is>
       </c>
-      <c r="W2" t="inlineStr"/>
-      <c r="X2" t="inlineStr"/>
       <c r="Y2" t="inlineStr"/>
       <c r="Z2" t="inlineStr"/>
       <c r="AA2" t="inlineStr"/>
@@ -784,110 +820,123 @@
       <c r="AC2" t="inlineStr"/>
       <c r="AD2" t="inlineStr"/>
       <c r="AE2" t="inlineStr"/>
-      <c r="AF2" t="inlineStr">
+      <c r="AF2" t="inlineStr"/>
+      <c r="AG2" t="inlineStr"/>
+      <c r="AH2" t="inlineStr">
         <is>
           <t>US</t>
         </is>
       </c>
-      <c r="AG2" t="n">
+      <c r="AI2" t="n">
         <v>25</v>
       </c>
-      <c r="AH2" t="n">
+      <c r="AJ2" t="n">
         <v>54</v>
       </c>
-      <c r="AI2" t="inlineStr"/>
-      <c r="AJ2" t="inlineStr"/>
       <c r="AK2" t="inlineStr"/>
-      <c r="AL2" t="inlineStr">
-        <is>
-          <t>1234567890</t>
-        </is>
-      </c>
+      <c r="AL2" t="inlineStr"/>
       <c r="AM2" t="inlineStr"/>
       <c r="AN2" t="inlineStr">
         <is>
-          <t>Ad A - Static</t>
-        </is>
-      </c>
-      <c r="AO2" t="inlineStr">
-        <is>
-          <t>https://example.com/creative-a.jpg</t>
-        </is>
-      </c>
+          <t>1234567890</t>
+        </is>
+      </c>
+      <c r="AO2" t="inlineStr"/>
       <c r="AP2" t="inlineStr"/>
       <c r="AQ2" t="inlineStr">
         <is>
+          <t>Ad A - Static</t>
+        </is>
+      </c>
+      <c r="AR2" t="inlineStr">
+        <is>
+          <t>https://example.com/creative-a.jpg</t>
+        </is>
+      </c>
+      <c r="AS2" t="inlineStr"/>
+      <c r="AT2" t="inlineStr">
+        <is>
           <t>Discover our new spring collection.</t>
         </is>
       </c>
-      <c r="AR2" t="inlineStr">
+      <c r="AU2" t="inlineStr">
         <is>
           <t>Spring is here</t>
         </is>
       </c>
-      <c r="AS2" t="inlineStr">
+      <c r="AV2" t="inlineStr">
         <is>
           <t>Shop the drop</t>
         </is>
       </c>
-      <c r="AT2" t="inlineStr">
+      <c r="AW2" t="inlineStr">
         <is>
           <t>https://example.com/spring</t>
         </is>
       </c>
-      <c r="AU2" t="inlineStr">
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>example.com</t>
+        </is>
+      </c>
+      <c r="AY2" t="inlineStr">
         <is>
           <t>utm_source=facebook&amp;utm_medium=cpc&amp;utm_campaign=spring</t>
         </is>
       </c>
-      <c r="AV2" t="inlineStr">
+      <c r="AZ2" t="inlineStr">
         <is>
           <t>SHOP_NOW</t>
         </is>
       </c>
-      <c r="AW2" t="inlineStr">
+      <c r="BA2" t="inlineStr"/>
+      <c r="BB2" t="inlineStr"/>
+      <c r="BC2" t="inlineStr">
         <is>
           <t>example.com</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="12">
-    <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid campaign_objective" promptTitle="campaign_objective" prompt="Choose from the list" type="list">
+  <dataValidations count="13">
+    <dataValidation sqref="C2:C500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid campaign_objective" promptTitle="campaign_objective" prompt="Choose from the list" type="list">
       <formula1>"OUTCOME_AWARENESS,OUTCOME_TRAFFIC,OUTCOME_ENGAGEMENT,OUTCOME_LEADS,OUTCOME_APP_PROMOTION,OUTCOME_SALES"</formula1>
     </dataValidation>
-    <dataValidation sqref="C2:C500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid buying_type" promptTitle="buying_type" prompt="Choose from the list" type="list">
+    <dataValidation sqref="D2:D500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid buying_type" promptTitle="buying_type" prompt="Choose from the list" type="list">
       <formula1>"AUCTION,RESERVED"</formula1>
     </dataValidation>
-    <dataValidation sqref="D2:D500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid special_ad_categories" promptTitle="special_ad_categories" prompt="Choose from the list" type="list">
+    <dataValidation sqref="E2:E500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid special_ad_categories" promptTitle="special_ad_categories" prompt="Choose from the list" type="list">
       <formula1>"NONE,HOUSING,CREDIT,EMPLOYMENT,ISSUES_ELECTIONS_POLITICS,ONLINE_GAMBLING_AND_GAMING,FINANCIAL_PRODUCTS_SERVICES"</formula1>
     </dataValidation>
-    <dataValidation sqref="G2:G500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid campaign_bid_strategy" promptTitle="campaign_bid_strategy" prompt="Choose from the list" type="list">
+    <dataValidation sqref="H2:H500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid campaign_bid_strategy" promptTitle="campaign_bid_strategy" prompt="Choose from the list" type="list">
       <formula1>"LOWEST_COST_WITHOUT_CAP,LOWEST_COST_WITH_BID_CAP,COST_CAP,LOWEST_COST_WITH_MIN_ROAS"</formula1>
     </dataValidation>
-    <dataValidation sqref="N2:N500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid bid_strategy" promptTitle="bid_strategy" prompt="Choose from the list" type="list">
+    <dataValidation sqref="P2:P500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid bid_strategy" promptTitle="bid_strategy" prompt="Choose from the list" type="list">
       <formula1>"LOWEST_COST_WITHOUT_CAP,LOWEST_COST_WITH_BID_CAP,COST_CAP,LOWEST_COST_WITH_MIN_ROAS"</formula1>
     </dataValidation>
-    <dataValidation sqref="S2:S500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid pacing_type" promptTitle="pacing_type" prompt="Choose from the list" type="list">
+    <dataValidation sqref="U2:U500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid pacing_type" promptTitle="pacing_type" prompt="Choose from the list" type="list">
       <formula1>",standard,no_pacing"</formula1>
     </dataValidation>
-    <dataValidation sqref="T2:T500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid billing_event" promptTitle="billing_event" prompt="Choose from the list" type="list">
+    <dataValidation sqref="V2:V500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid billing_event" promptTitle="billing_event" prompt="Choose from the list" type="list">
       <formula1>"IMPRESSIONS,LINK_CLICKS,POST_ENGAGEMENT,VIDEO_VIEWS,THRUPLAY"</formula1>
     </dataValidation>
-    <dataValidation sqref="U2:U500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid optimization_goal" promptTitle="optimization_goal" prompt="Choose from the list" type="list">
+    <dataValidation sqref="W2:W500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid optimization_goal" promptTitle="optimization_goal" prompt="Choose from the list" type="list">
       <formula1>"REACH,IMPRESSIONS,LINK_CLICKS,LANDING_PAGE_VIEWS,POST_ENGAGEMENT,PAGE_LIKES,VIDEO_VIEWS,THRUPLAY,OFFSITE_CONVERSIONS,VALUE,LEAD_GENERATION,QUALITY_LEAD,CONVERSATIONS,APP_INSTALLS,AD_RECALL_LIFT"</formula1>
     </dataValidation>
-    <dataValidation sqref="V2:V500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid destination_type" promptTitle="destination_type" prompt="Choose from the list" type="list">
+    <dataValidation sqref="X2:X500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid destination_type" promptTitle="destination_type" prompt="Choose from the list" type="list">
       <formula1>"WEBSITE,APP,MESSENGER,INSTAGRAM_DIRECT,WHATSAPP,FACEBOOK,ON_AD,ON_POST,ON_PAGE,ON_EVENT,ON_VIDEO,SHOP_AUTOMATIC"</formula1>
     </dataValidation>
-    <dataValidation sqref="Z2:Z500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid custom_event_type" promptTitle="custom_event_type" prompt="Choose from the list" type="list">
+    <dataValidation sqref="AB2:AB500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid custom_event_type" promptTitle="custom_event_type" prompt="Choose from the list" type="list">
       <formula1>",PURCHASE,LEAD,COMPLETE_REGISTRATION,ADD_TO_CART,INITIATE_CHECKOUT,ADD_PAYMENT_INFO,VIEW_CONTENT,SEARCH,SUBSCRIBE,CONTACT,DONATE,OTHER"</formula1>
     </dataValidation>
-    <dataValidation sqref="AI2:AI500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid genders" promptTitle="genders" prompt="Choose from the list" type="list">
+    <dataValidation sqref="AK2:AK500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid genders" promptTitle="genders" prompt="Choose from the list" type="list">
       <formula1>",1,2,1,2"</formula1>
     </dataValidation>
-    <dataValidation sqref="AV2:AV500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid cta" promptTitle="cta" prompt="Choose from the list" type="list">
+    <dataValidation sqref="AZ2:AZ500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid cta" promptTitle="cta" prompt="Choose from the list" type="list">
       <formula1>"SHOP_NOW,LEARN_MORE,SIGN_UP,SUBSCRIBE,DOWNLOAD,BOOK_TRAVEL,CONTACT_US,GET_OFFER,GET_QUOTE,APPLY_NOW,ORDER_NOW,DONATE_NOW,INSTALL_APP,USE_APP,WATCH_MORE,LISTEN_NOW,SEND_MESSAGE,MESSAGE_PAGE,GET_DIRECTIONS,CALL_NOW,NO_BUTTON"</formula1>
+    </dataValidation>
+    <dataValidation sqref="BA2:BA500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid browser_addon" promptTitle="browser_addon" prompt="Choose from the list" type="list">
+      <formula1>",NONE,CALL,MESSENGER,WHATSAPP"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Rename instagram_actor_id template column to instagram_user_id
Matches the current Meta API field name. The API value the column
maps to was already instagram_user_id (Meta renamed the field
upstream); this just makes the spreadsheet column name match.
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -456,7 +456,7 @@
     <col width="30" customWidth="1" min="38" max="38"/>
     <col width="30" customWidth="1" min="39" max="39"/>
     <col width="14" customWidth="1" min="40" max="40"/>
-    <col width="20" customWidth="1" min="41" max="41"/>
+    <col width="19" customWidth="1" min="41" max="41"/>
     <col width="17" customWidth="1" min="42" max="42"/>
     <col width="14" customWidth="1" min="43" max="43"/>
     <col width="14" customWidth="1" min="44" max="44"/>
@@ -676,7 +676,7 @@
       </c>
       <c r="AO1" t="inlineStr">
         <is>
-          <t>instagram_actor_id</t>
+          <t>instagram_user_id</t>
         </is>
       </c>
       <c r="AP1" t="inlineStr">

</xml_diff>

<commit_message>
Add advantage_plus_creative master switch (Standard Enhancements)
Maps to the ad creative's degrees_of_freedom_spec.creative_features
_spec.standard_enhancements. ENABLED sets enroll_status=OPT_IN
(turns on Advantage+ creative enhancements like image touch-ups,
text improvements, etc.), DISABLED sets OPT_OUT, blank leaves it
at the account default. For per-feature opt-outs (e.g. turn off
just 'Add product tags'), users still need to edit individual
toggles in Ads Manager after the upload.
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BD2"/>
+  <dimension ref="A1:BE2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -472,6 +472,7 @@
     <col width="15" customWidth="1" min="54" max="54"/>
     <col width="14" customWidth="1" min="55" max="55"/>
     <col width="19" customWidth="1" min="56" max="56"/>
+    <col width="25" customWidth="1" min="57" max="57"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -753,6 +754,11 @@
       <c r="BD1" t="inlineStr">
         <is>
           <t>conversion_domain</t>
+        </is>
+      </c>
+      <c r="BE1" t="inlineStr">
+        <is>
+          <t>advantage_plus_creative</t>
         </is>
       </c>
     </row>
@@ -903,9 +909,10 @@
           <t>example.com</t>
         </is>
       </c>
+      <c r="BE2" t="inlineStr"/>
     </row>
   </sheetData>
-  <dataValidations count="13">
+  <dataValidations count="14">
     <dataValidation sqref="C2:C500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid campaign_objective" promptTitle="campaign_objective" prompt="Choose from the list" type="list">
       <formula1>"OUTCOME_AWARENESS,OUTCOME_TRAFFIC,OUTCOME_ENGAGEMENT,OUTCOME_LEADS,OUTCOME_APP_PROMOTION,OUTCOME_SALES"</formula1>
     </dataValidation>
@@ -944,6 +951,9 @@
     </dataValidation>
     <dataValidation sqref="BB2:BB500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid browser_addon" promptTitle="browser_addon" prompt="Choose from the list" type="list">
       <formula1>",NONE,CALL,MESSENGER,WHATSAPP"</formula1>
+    </dataValidation>
+    <dataValidation sqref="BE2:BE500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid advantage_plus_creative" promptTitle="advantage_plus_creative" prompt="Choose from the list" type="list">
+      <formula1>",ENABLED,DISABLED"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add per-feature columns for Advantage+ creative enhancements
Seven new columns each map to a specific Meta API feature key in
degrees_of_freedom_spec.creative_features_spec, with dropdown
values blank / OPT_IN / OPT_OUT:

  adv_image_animation         -> IMAGE_ANIMATION
  adv_image_touchups          -> IMAGE_TOUCHUPS
  adv_text_generation         -> TEXT_GENERATION
  adv_text_overlay_translation -> TEXT_OVERLAY_TRANSLATION
  adv_ig_video_subtitle       -> IG_VIDEO_NATIVE_SUBTITLE
  adv_music                   -> MUSIC
  adv_profile_card            -> PROFILE_CARD

These layer on top of the existing advantage_plus_creative master
switch — set the master to ENABLED for the broad baseline, then
override individual features per ad.
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BE2"/>
+  <dimension ref="A1:BL2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -473,6 +473,13 @@
     <col width="14" customWidth="1" min="55" max="55"/>
     <col width="19" customWidth="1" min="56" max="56"/>
     <col width="25" customWidth="1" min="57" max="57"/>
+    <col width="21" customWidth="1" min="58" max="58"/>
+    <col width="20" customWidth="1" min="59" max="59"/>
+    <col width="21" customWidth="1" min="60" max="60"/>
+    <col width="30" customWidth="1" min="61" max="61"/>
+    <col width="23" customWidth="1" min="62" max="62"/>
+    <col width="14" customWidth="1" min="63" max="63"/>
+    <col width="18" customWidth="1" min="64" max="64"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -759,6 +766,41 @@
       <c r="BE1" t="inlineStr">
         <is>
           <t>advantage_plus_creative</t>
+        </is>
+      </c>
+      <c r="BF1" t="inlineStr">
+        <is>
+          <t>adv_image_animation</t>
+        </is>
+      </c>
+      <c r="BG1" t="inlineStr">
+        <is>
+          <t>adv_image_touchups</t>
+        </is>
+      </c>
+      <c r="BH1" t="inlineStr">
+        <is>
+          <t>adv_text_generation</t>
+        </is>
+      </c>
+      <c r="BI1" t="inlineStr">
+        <is>
+          <t>adv_text_overlay_translation</t>
+        </is>
+      </c>
+      <c r="BJ1" t="inlineStr">
+        <is>
+          <t>adv_ig_video_subtitle</t>
+        </is>
+      </c>
+      <c r="BK1" t="inlineStr">
+        <is>
+          <t>adv_music</t>
+        </is>
+      </c>
+      <c r="BL1" t="inlineStr">
+        <is>
+          <t>adv_profile_card</t>
         </is>
       </c>
     </row>
@@ -910,9 +952,16 @@
         </is>
       </c>
       <c r="BE2" t="inlineStr"/>
+      <c r="BF2" t="inlineStr"/>
+      <c r="BG2" t="inlineStr"/>
+      <c r="BH2" t="inlineStr"/>
+      <c r="BI2" t="inlineStr"/>
+      <c r="BJ2" t="inlineStr"/>
+      <c r="BK2" t="inlineStr"/>
+      <c r="BL2" t="inlineStr"/>
     </row>
   </sheetData>
-  <dataValidations count="14">
+  <dataValidations count="21">
     <dataValidation sqref="C2:C500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid campaign_objective" promptTitle="campaign_objective" prompt="Choose from the list" type="list">
       <formula1>"OUTCOME_AWARENESS,OUTCOME_TRAFFIC,OUTCOME_ENGAGEMENT,OUTCOME_LEADS,OUTCOME_APP_PROMOTION,OUTCOME_SALES"</formula1>
     </dataValidation>
@@ -954,6 +1003,27 @@
     </dataValidation>
     <dataValidation sqref="BE2:BE500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid advantage_plus_creative" promptTitle="advantage_plus_creative" prompt="Choose from the list" type="list">
       <formula1>",ENABLED,DISABLED"</formula1>
+    </dataValidation>
+    <dataValidation sqref="BF2:BF500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_image_animation" promptTitle="adv_image_animation" prompt="Choose from the list" type="list">
+      <formula1>",OPT_IN,OPT_OUT"</formula1>
+    </dataValidation>
+    <dataValidation sqref="BG2:BG500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_image_touchups" promptTitle="adv_image_touchups" prompt="Choose from the list" type="list">
+      <formula1>",OPT_IN,OPT_OUT"</formula1>
+    </dataValidation>
+    <dataValidation sqref="BH2:BH500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_text_generation" promptTitle="adv_text_generation" prompt="Choose from the list" type="list">
+      <formula1>",OPT_IN,OPT_OUT"</formula1>
+    </dataValidation>
+    <dataValidation sqref="BI2:BI500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_text_overlay_translation" promptTitle="adv_text_overlay_translation" prompt="Choose from the list" type="list">
+      <formula1>",OPT_IN,OPT_OUT"</formula1>
+    </dataValidation>
+    <dataValidation sqref="BJ2:BJ500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_ig_video_subtitle" promptTitle="adv_ig_video_subtitle" prompt="Choose from the list" type="list">
+      <formula1>",OPT_IN,OPT_OUT"</formula1>
+    </dataValidation>
+    <dataValidation sqref="BK2:BK500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_music" promptTitle="adv_music" prompt="Choose from the list" type="list">
+      <formula1>",OPT_IN,OPT_OUT"</formula1>
+    </dataValidation>
+    <dataValidation sqref="BL2:BL500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_profile_card" promptTitle="adv_profile_card" prompt="Choose from the list" type="list">
+      <formula1>",OPT_IN,OPT_OUT"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Switch Advantage+ dropdowns from OPT_IN/OPT_OUT to ON/OFF
User-facing dropdowns now use plain ON/OFF instead of the Meta API
strings; the script translates ON->OPT_IN and OFF->OPT_OUT before
sending. Master switch likewise uses ON/OFF instead of
ENABLED/DISABLED for consistency. CSV cell values stay blank by
default so no template.csv change is needed.
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -1051,49 +1051,49 @@
       <formula1>",NONE,CALL,MESSENGER,WHATSAPP"</formula1>
     </dataValidation>
     <dataValidation sqref="BE2:BE500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid advantage_plus_creative" promptTitle="advantage_plus_creative" prompt="Choose from the list" type="list">
-      <formula1>",ENABLED,DISABLED"</formula1>
+      <formula1>",ON,OFF"</formula1>
     </dataValidation>
     <dataValidation sqref="BF2:BF500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_add_overlays" promptTitle="adv_add_overlays" prompt="Choose from the list" type="list">
-      <formula1>",OPT_IN,OPT_OUT"</formula1>
+      <formula1>",ON,OFF"</formula1>
     </dataValidation>
     <dataValidation sqref="BG2:BG500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_image_touchups" promptTitle="adv_image_touchups" prompt="Choose from the list" type="list">
-      <formula1>",OPT_IN,OPT_OUT"</formula1>
+      <formula1>",ON,OFF"</formula1>
     </dataValidation>
     <dataValidation sqref="BH2:BH500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_music" promptTitle="adv_music" prompt="Choose from the list" type="list">
-      <formula1>",OPT_IN,OPT_OUT"</formula1>
+      <formula1>",ON,OFF"</formula1>
     </dataValidation>
     <dataValidation sqref="BI2:BI500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_text_generation" promptTitle="adv_text_generation" prompt="Choose from the list" type="list">
-      <formula1>",OPT_IN,OPT_OUT"</formula1>
+      <formula1>",ON,OFF"</formula1>
     </dataValidation>
     <dataValidation sqref="BJ2:BJ500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_image_animation" promptTitle="adv_image_animation" prompt="Choose from the list" type="list">
-      <formula1>",OPT_IN,OPT_OUT"</formula1>
+      <formula1>",ON,OFF"</formula1>
     </dataValidation>
     <dataValidation sqref="BK2:BK500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_product_tags" promptTitle="adv_product_tags" prompt="Choose from the list" type="list">
-      <formula1>",OPT_IN,OPT_OUT"</formula1>
+      <formula1>",ON,OFF"</formula1>
     </dataValidation>
     <dataValidation sqref="BL2:BL500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_relevant_comments" promptTitle="adv_relevant_comments" prompt="Choose from the list" type="list">
-      <formula1>",OPT_IN,OPT_OUT"</formula1>
+      <formula1>",ON,OFF"</formula1>
     </dataValidation>
     <dataValidation sqref="BM2:BM500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_enhance_cta" promptTitle="adv_enhance_cta" prompt="Choose from the list" type="list">
-      <formula1>",OPT_IN,OPT_OUT"</formula1>
+      <formula1>",ON,OFF"</formula1>
     </dataValidation>
     <dataValidation sqref="BN2:BN500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_brightness_contrast" promptTitle="adv_brightness_contrast" prompt="Choose from the list" type="list">
-      <formula1>",OPT_IN,OPT_OUT"</formula1>
+      <formula1>",ON,OFF"</formula1>
     </dataValidation>
     <dataValidation sqref="BO2:BO500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_reveal_details" promptTitle="adv_reveal_details" prompt="Choose from the list" type="list">
-      <formula1>",OPT_IN,OPT_OUT"</formula1>
+      <formula1>",ON,OFF"</formula1>
     </dataValidation>
     <dataValidation sqref="BP2:BP500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_spotlights" promptTitle="adv_spotlights" prompt="Choose from the list" type="list">
-      <formula1>",OPT_IN,OPT_OUT"</formula1>
+      <formula1>",ON,OFF"</formula1>
     </dataValidation>
     <dataValidation sqref="BQ2:BQ500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_text_overlay_translation" promptTitle="adv_text_overlay_translation" prompt="Choose from the list" type="list">
-      <formula1>",OPT_IN,OPT_OUT"</formula1>
+      <formula1>",ON,OFF"</formula1>
     </dataValidation>
     <dataValidation sqref="BR2:BR500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_ig_video_subtitle" promptTitle="adv_ig_video_subtitle" prompt="Choose from the list" type="list">
-      <formula1>",OPT_IN,OPT_OUT"</formula1>
+      <formula1>",ON,OFF"</formula1>
     </dataValidation>
     <dataValidation sqref="BS2:BS500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_profile_card" promptTitle="adv_profile_card" prompt="Choose from the list" type="list">
-      <formula1>",OPT_IN,OPT_OUT"</formula1>
+      <formula1>",ON,OFF"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Rewrite dropdown generation to use a hidden _options sheet
Inline 'a,b,c' DataValidation formulas are unreliable across Excel /
Google Sheets / Numbers — Sheets in particular silently drops them
when the list begins with an empty option (',ON,OFF') or when the
formula string is long. The new approach stores each dropdown's
values down a column of a hidden '_options' sheet and references
them by absolute range (e.g. ='_options'!$A$1:$A$6), which all
three tools render reliably.
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="ads" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="_options" sheetId="2" state="hidden" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1012,90 +1013,781 @@
   </sheetData>
   <dataValidations count="28">
     <dataValidation sqref="C2:C500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid campaign_objective" promptTitle="campaign_objective" prompt="Choose from the list" type="list">
-      <formula1>"OUTCOME_AWARENESS,OUTCOME_TRAFFIC,OUTCOME_ENGAGEMENT,OUTCOME_LEADS,OUTCOME_APP_PROMOTION,OUTCOME_SALES"</formula1>
+      <formula1>='_options'!$A$1:$A$6</formula1>
     </dataValidation>
     <dataValidation sqref="D2:D500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid buying_type" promptTitle="buying_type" prompt="Choose from the list" type="list">
-      <formula1>"AUCTION,RESERVED"</formula1>
+      <formula1>='_options'!$B$1:$B$2</formula1>
     </dataValidation>
     <dataValidation sqref="E2:E500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid special_ad_categories" promptTitle="special_ad_categories" prompt="Choose from the list" type="list">
-      <formula1>"NONE,HOUSING,CREDIT,EMPLOYMENT,ISSUES_ELECTIONS_POLITICS,ONLINE_GAMBLING_AND_GAMING,FINANCIAL_PRODUCTS_SERVICES"</formula1>
+      <formula1>='_options'!$C$1:$C$7</formula1>
     </dataValidation>
     <dataValidation sqref="H2:H500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid campaign_bid_strategy" promptTitle="campaign_bid_strategy" prompt="Choose from the list" type="list">
-      <formula1>"LOWEST_COST_WITHOUT_CAP,LOWEST_COST_WITH_BID_CAP,COST_CAP,LOWEST_COST_WITH_MIN_ROAS"</formula1>
+      <formula1>='_options'!$D$1:$D$4</formula1>
     </dataValidation>
     <dataValidation sqref="P2:P500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid bid_strategy" promptTitle="bid_strategy" prompt="Choose from the list" type="list">
-      <formula1>"LOWEST_COST_WITHOUT_CAP,LOWEST_COST_WITH_BID_CAP,COST_CAP,LOWEST_COST_WITH_MIN_ROAS"</formula1>
+      <formula1>='_options'!$E$1:$E$4</formula1>
     </dataValidation>
     <dataValidation sqref="U2:U500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid pacing_type" promptTitle="pacing_type" prompt="Choose from the list" type="list">
-      <formula1>",standard,no_pacing"</formula1>
+      <formula1>='_options'!$F$1:$F$2</formula1>
     </dataValidation>
     <dataValidation sqref="V2:V500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid billing_event" promptTitle="billing_event" prompt="Choose from the list" type="list">
-      <formula1>"IMPRESSIONS,LINK_CLICKS,POST_ENGAGEMENT,VIDEO_VIEWS,THRUPLAY"</formula1>
+      <formula1>='_options'!$G$1:$G$5</formula1>
     </dataValidation>
     <dataValidation sqref="W2:W500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid optimization_goal" promptTitle="optimization_goal" prompt="Choose from the list" type="list">
-      <formula1>"REACH,IMPRESSIONS,LINK_CLICKS,LANDING_PAGE_VIEWS,POST_ENGAGEMENT,PAGE_LIKES,VIDEO_VIEWS,THRUPLAY,OFFSITE_CONVERSIONS,VALUE,LEAD_GENERATION,QUALITY_LEAD,CONVERSATIONS,APP_INSTALLS,AD_RECALL_LIFT"</formula1>
+      <formula1>='_options'!$H$1:$H$15</formula1>
     </dataValidation>
     <dataValidation sqref="X2:X500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid destination_type" promptTitle="destination_type" prompt="Choose from the list" type="list">
-      <formula1>"WEBSITE,APP,MESSENGER,INSTAGRAM_DIRECT,WHATSAPP,FACEBOOK,ON_AD,ON_POST,ON_PAGE,ON_EVENT,ON_VIDEO,SHOP_AUTOMATIC"</formula1>
+      <formula1>='_options'!$I$1:$I$12</formula1>
     </dataValidation>
     <dataValidation sqref="AB2:AB500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid custom_event_type" promptTitle="custom_event_type" prompt="Choose from the list" type="list">
-      <formula1>",PURCHASE,LEAD,COMPLETE_REGISTRATION,ADD_TO_CART,INITIATE_CHECKOUT,ADD_PAYMENT_INFO,VIEW_CONTENT,SEARCH,SUBSCRIBE,CONTACT,DONATE,OTHER"</formula1>
+      <formula1>='_options'!$J$1:$J$12</formula1>
     </dataValidation>
     <dataValidation sqref="AK2:AK500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid genders" promptTitle="genders" prompt="Choose from the list" type="list">
-      <formula1>",1,2,1,2"</formula1>
+      <formula1>='_options'!$K$1:$K$3</formula1>
     </dataValidation>
     <dataValidation sqref="BA2:BA500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid cta" promptTitle="cta" prompt="Choose from the list" type="list">
-      <formula1>"SHOP_NOW,LEARN_MORE,SIGN_UP,SUBSCRIBE,DOWNLOAD,BOOK_TRAVEL,CONTACT_US,GET_OFFER,GET_QUOTE,APPLY_NOW,ORDER_NOW,DONATE_NOW,INSTALL_APP,USE_APP,WATCH_MORE,LISTEN_NOW,SEND_MESSAGE,MESSAGE_PAGE,GET_DIRECTIONS,CALL_NOW,NO_BUTTON"</formula1>
+      <formula1>='_options'!$L$1:$L$21</formula1>
     </dataValidation>
     <dataValidation sqref="BB2:BB500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid browser_addon" promptTitle="browser_addon" prompt="Choose from the list" type="list">
-      <formula1>",NONE,CALL,MESSENGER,WHATSAPP"</formula1>
+      <formula1>='_options'!$M$1:$M$4</formula1>
     </dataValidation>
     <dataValidation sqref="BE2:BE500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid advantage_plus_creative" promptTitle="advantage_plus_creative" prompt="Choose from the list" type="list">
-      <formula1>",ON,OFF"</formula1>
+      <formula1>='_options'!$N$1:$N$2</formula1>
     </dataValidation>
     <dataValidation sqref="BF2:BF500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_add_overlays" promptTitle="adv_add_overlays" prompt="Choose from the list" type="list">
-      <formula1>",ON,OFF"</formula1>
+      <formula1>='_options'!$O$1:$O$2</formula1>
     </dataValidation>
     <dataValidation sqref="BG2:BG500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_image_touchups" promptTitle="adv_image_touchups" prompt="Choose from the list" type="list">
-      <formula1>",ON,OFF"</formula1>
+      <formula1>='_options'!$P$1:$P$2</formula1>
     </dataValidation>
     <dataValidation sqref="BH2:BH500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_music" promptTitle="adv_music" prompt="Choose from the list" type="list">
-      <formula1>",ON,OFF"</formula1>
+      <formula1>='_options'!$Q$1:$Q$2</formula1>
     </dataValidation>
     <dataValidation sqref="BI2:BI500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_text_generation" promptTitle="adv_text_generation" prompt="Choose from the list" type="list">
-      <formula1>",ON,OFF"</formula1>
+      <formula1>='_options'!$R$1:$R$2</formula1>
     </dataValidation>
     <dataValidation sqref="BJ2:BJ500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_image_animation" promptTitle="adv_image_animation" prompt="Choose from the list" type="list">
-      <formula1>",ON,OFF"</formula1>
+      <formula1>='_options'!$S$1:$S$2</formula1>
     </dataValidation>
     <dataValidation sqref="BK2:BK500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_product_tags" promptTitle="adv_product_tags" prompt="Choose from the list" type="list">
-      <formula1>",ON,OFF"</formula1>
+      <formula1>='_options'!$T$1:$T$2</formula1>
     </dataValidation>
     <dataValidation sqref="BL2:BL500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_relevant_comments" promptTitle="adv_relevant_comments" prompt="Choose from the list" type="list">
-      <formula1>",ON,OFF"</formula1>
+      <formula1>='_options'!$U$1:$U$2</formula1>
     </dataValidation>
     <dataValidation sqref="BM2:BM500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_enhance_cta" promptTitle="adv_enhance_cta" prompt="Choose from the list" type="list">
-      <formula1>",ON,OFF"</formula1>
+      <formula1>='_options'!$V$1:$V$2</formula1>
     </dataValidation>
     <dataValidation sqref="BN2:BN500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_brightness_contrast" promptTitle="adv_brightness_contrast" prompt="Choose from the list" type="list">
-      <formula1>",ON,OFF"</formula1>
+      <formula1>='_options'!$W$1:$W$2</formula1>
     </dataValidation>
     <dataValidation sqref="BO2:BO500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_reveal_details" promptTitle="adv_reveal_details" prompt="Choose from the list" type="list">
-      <formula1>",ON,OFF"</formula1>
+      <formula1>='_options'!$X$1:$X$2</formula1>
     </dataValidation>
     <dataValidation sqref="BP2:BP500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_spotlights" promptTitle="adv_spotlights" prompt="Choose from the list" type="list">
-      <formula1>",ON,OFF"</formula1>
+      <formula1>='_options'!$Y$1:$Y$2</formula1>
     </dataValidation>
     <dataValidation sqref="BQ2:BQ500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_text_overlay_translation" promptTitle="adv_text_overlay_translation" prompt="Choose from the list" type="list">
-      <formula1>",ON,OFF"</formula1>
+      <formula1>='_options'!$Z$1:$Z$2</formula1>
     </dataValidation>
     <dataValidation sqref="BR2:BR500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_ig_video_subtitle" promptTitle="adv_ig_video_subtitle" prompt="Choose from the list" type="list">
-      <formula1>",ON,OFF"</formula1>
+      <formula1>='_options'!$AA$1:$AA$2</formula1>
     </dataValidation>
     <dataValidation sqref="BS2:BS500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_profile_card" promptTitle="adv_profile_card" prompt="Choose from the list" type="list">
-      <formula1>",ON,OFF"</formula1>
+      <formula1>='_options'!$AB$1:$AB$2</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:AB21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>OUTCOME_AWARENESS</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>AUCTION</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>LOWEST_COST_WITHOUT_CAP</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>LOWEST_COST_WITHOUT_CAP</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>IMPRESSIONS</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>REACH</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>WEBSITE</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>PURCHASE</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>SHOP_NOW</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>OUTCOME_TRAFFIC</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>RESERVED</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>HOUSING</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>LOWEST_COST_WITH_BID_CAP</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>LOWEST_COST_WITH_BID_CAP</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>no_pacing</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>LINK_CLICKS</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>IMPRESSIONS</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>APP</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>LEAD</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>LEARN_MORE</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>OUTCOME_ENGAGEMENT</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CREDIT</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>COST_CAP</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>COST_CAP</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>POST_ENGAGEMENT</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>LINK_CLICKS</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>MESSENGER</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>COMPLETE_REGISTRATION</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>1,2</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>SIGN_UP</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>MESSENGER</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>OUTCOME_LEADS</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>EMPLOYMENT</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>LOWEST_COST_WITH_MIN_ROAS</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>LOWEST_COST_WITH_MIN_ROAS</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>VIDEO_VIEWS</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>LANDING_PAGE_VIEWS</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>INSTAGRAM_DIRECT</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>ADD_TO_CART</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>SUBSCRIBE</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>WHATSAPP</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>OUTCOME_APP_PROMOTION</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>ISSUES_ELECTIONS_POLITICS</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>THRUPLAY</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>POST_ENGAGEMENT</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>WHATSAPP</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>INITIATE_CHECKOUT</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>DOWNLOAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>OUTCOME_SALES</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>ONLINE_GAMBLING_AND_GAMING</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>PAGE_LIKES</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>FACEBOOK</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>ADD_PAYMENT_INFO</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>BOOK_TRAVEL</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>FINANCIAL_PRODUCTS_SERVICES</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>VIDEO_VIEWS</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>ON_AD</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>VIEW_CONTENT</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>CONTACT_US</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>THRUPLAY</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>ON_POST</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>SEARCH</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>GET_OFFER</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>OFFSITE_CONVERSIONS</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>ON_PAGE</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>SUBSCRIBE</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>GET_QUOTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>VALUE</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>ON_EVENT</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>CONTACT</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>APPLY_NOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>LEAD_GENERATION</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>ON_VIDEO</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>DONATE</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>ORDER_NOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>QUALITY_LEAD</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>SHOP_AUTOMATIC</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>OTHER</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>DONATE_NOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>CONVERSATIONS</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>INSTALL_APP</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>APP_INSTALLS</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>USE_APP</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>AD_RECALL_LIFT</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>WATCH_MORE</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>LISTEN_NOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>SEND_MESSAGE</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>MESSAGE_PAGE</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>GET_DIRECTIONS</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>CALL_NOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>NO_BUTTON</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Use named ranges for dropdowns; visible _options sheet; 1 sample row
- Dropdowns now reference workbook-level named ranges (e.g.
  'cta_options') instead of inline 'a,b,c' formulas. This is the
  format Google Sheets / Excel online / Numbers all accept
  consistently.
- _options sheet is no longer hidden — user can see the dropdown
  values exist if any tool fails to render the validation arrow.
- template.csv and template.xlsx both trimmed to one example row.
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -8,9 +8,38 @@
   </bookViews>
   <sheets>
     <sheet name="ads" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="_options" sheetId="2" state="hidden" r:id="rId2"/>
+    <sheet name="_options" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="campaign_objective_options">'_options'!$A$2:$A$7</definedName>
+    <definedName name="buying_type_options">'_options'!$B$2:$B$3</definedName>
+    <definedName name="special_ad_categories_options">'_options'!$C$2:$C$8</definedName>
+    <definedName name="campaign_bid_strategy_options">'_options'!$D$2:$D$5</definedName>
+    <definedName name="bid_strategy_options">'_options'!$E$2:$E$5</definedName>
+    <definedName name="pacing_type_options">'_options'!$F$2:$F$3</definedName>
+    <definedName name="billing_event_options">'_options'!$G$2:$G$6</definedName>
+    <definedName name="optimization_goal_options">'_options'!$H$2:$H$16</definedName>
+    <definedName name="destination_type_options">'_options'!$I$2:$I$13</definedName>
+    <definedName name="custom_event_type_options">'_options'!$J$2:$J$13</definedName>
+    <definedName name="genders_options">'_options'!$K$2:$K$4</definedName>
+    <definedName name="cta_options">'_options'!$L$2:$L$22</definedName>
+    <definedName name="browser_addon_options">'_options'!$M$2:$M$5</definedName>
+    <definedName name="advantage_plus_creative_options">'_options'!$N$2:$N$3</definedName>
+    <definedName name="adv_add_overlays_options">'_options'!$O$2:$O$3</definedName>
+    <definedName name="adv_image_touchups_options">'_options'!$P$2:$P$3</definedName>
+    <definedName name="adv_music_options">'_options'!$Q$2:$Q$3</definedName>
+    <definedName name="adv_text_generation_options">'_options'!$R$2:$R$3</definedName>
+    <definedName name="adv_image_animation_options">'_options'!$S$2:$S$3</definedName>
+    <definedName name="adv_product_tags_options">'_options'!$T$2:$T$3</definedName>
+    <definedName name="adv_relevant_comments_options">'_options'!$U$2:$U$3</definedName>
+    <definedName name="adv_enhance_cta_options">'_options'!$V$2:$V$3</definedName>
+    <definedName name="adv_brightness_contrast_options">'_options'!$W$2:$W$3</definedName>
+    <definedName name="adv_reveal_details_options">'_options'!$X$2:$X$3</definedName>
+    <definedName name="adv_spotlights_options">'_options'!$Y$2:$Y$3</definedName>
+    <definedName name="adv_text_overlay_translation_options">'_options'!$Z$2:$Z$3</definedName>
+    <definedName name="adv_ig_video_subtitle_options">'_options'!$AA$2:$AA$3</definedName>
+    <definedName name="adv_profile_card_options">'_options'!$AB$2:$AB$3</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -851,7 +880,7 @@
       <c r="A2" t="inlineStr"/>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Spring Launch</t>
+          <t>My First Campaign</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -878,7 +907,7 @@
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>US Broad 25-54</t>
+          <t>My First Ad Set</t>
         </is>
       </c>
       <c r="N2" t="n">
@@ -942,34 +971,34 @@
       <c r="AP2" t="inlineStr"/>
       <c r="AQ2" t="inlineStr">
         <is>
-          <t>Ad A - Static</t>
+          <t>My First Ad</t>
         </is>
       </c>
       <c r="AR2" t="inlineStr">
         <is>
-          <t>https://example.com/creative-a.jpg</t>
+          <t>https://example.com/image.jpg</t>
         </is>
       </c>
       <c r="AS2" t="inlineStr"/>
       <c r="AT2" t="inlineStr"/>
       <c r="AU2" t="inlineStr">
         <is>
-          <t>Discover our new spring collection.</t>
+          <t>Body copy goes here.</t>
         </is>
       </c>
       <c r="AV2" t="inlineStr">
         <is>
-          <t>Spring is here</t>
+          <t>Your headline</t>
         </is>
       </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>Shop the drop</t>
+          <t>Short description.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>https://example.com/spring</t>
+          <t>https://example.com/landing</t>
         </is>
       </c>
       <c r="AY2" t="inlineStr">
@@ -977,11 +1006,7 @@
           <t>example.com</t>
         </is>
       </c>
-      <c r="AZ2" t="inlineStr">
-        <is>
-          <t>utm_source=facebook&amp;utm_medium=cpc&amp;utm_campaign=spring</t>
-        </is>
-      </c>
+      <c r="AZ2" t="inlineStr"/>
       <c r="BA2" t="inlineStr">
         <is>
           <t>SHOP_NOW</t>
@@ -1013,88 +1038,88 @@
   </sheetData>
   <dataValidations count="28">
     <dataValidation sqref="C2:C500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid campaign_objective" promptTitle="campaign_objective" prompt="Choose from the list" type="list">
-      <formula1>='_options'!$A$1:$A$6</formula1>
+      <formula1>campaign_objective_options</formula1>
     </dataValidation>
     <dataValidation sqref="D2:D500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid buying_type" promptTitle="buying_type" prompt="Choose from the list" type="list">
-      <formula1>='_options'!$B$1:$B$2</formula1>
+      <formula1>buying_type_options</formula1>
     </dataValidation>
     <dataValidation sqref="E2:E500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid special_ad_categories" promptTitle="special_ad_categories" prompt="Choose from the list" type="list">
-      <formula1>='_options'!$C$1:$C$7</formula1>
+      <formula1>special_ad_categories_options</formula1>
     </dataValidation>
     <dataValidation sqref="H2:H500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid campaign_bid_strategy" promptTitle="campaign_bid_strategy" prompt="Choose from the list" type="list">
-      <formula1>='_options'!$D$1:$D$4</formula1>
+      <formula1>campaign_bid_strategy_options</formula1>
     </dataValidation>
     <dataValidation sqref="P2:P500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid bid_strategy" promptTitle="bid_strategy" prompt="Choose from the list" type="list">
-      <formula1>='_options'!$E$1:$E$4</formula1>
+      <formula1>bid_strategy_options</formula1>
     </dataValidation>
     <dataValidation sqref="U2:U500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid pacing_type" promptTitle="pacing_type" prompt="Choose from the list" type="list">
-      <formula1>='_options'!$F$1:$F$2</formula1>
+      <formula1>pacing_type_options</formula1>
     </dataValidation>
     <dataValidation sqref="V2:V500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid billing_event" promptTitle="billing_event" prompt="Choose from the list" type="list">
-      <formula1>='_options'!$G$1:$G$5</formula1>
+      <formula1>billing_event_options</formula1>
     </dataValidation>
     <dataValidation sqref="W2:W500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid optimization_goal" promptTitle="optimization_goal" prompt="Choose from the list" type="list">
-      <formula1>='_options'!$H$1:$H$15</formula1>
+      <formula1>optimization_goal_options</formula1>
     </dataValidation>
     <dataValidation sqref="X2:X500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid destination_type" promptTitle="destination_type" prompt="Choose from the list" type="list">
-      <formula1>='_options'!$I$1:$I$12</formula1>
+      <formula1>destination_type_options</formula1>
     </dataValidation>
     <dataValidation sqref="AB2:AB500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid custom_event_type" promptTitle="custom_event_type" prompt="Choose from the list" type="list">
-      <formula1>='_options'!$J$1:$J$12</formula1>
+      <formula1>custom_event_type_options</formula1>
     </dataValidation>
     <dataValidation sqref="AK2:AK500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid genders" promptTitle="genders" prompt="Choose from the list" type="list">
-      <formula1>='_options'!$K$1:$K$3</formula1>
+      <formula1>genders_options</formula1>
     </dataValidation>
     <dataValidation sqref="BA2:BA500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid cta" promptTitle="cta" prompt="Choose from the list" type="list">
-      <formula1>='_options'!$L$1:$L$21</formula1>
+      <formula1>cta_options</formula1>
     </dataValidation>
     <dataValidation sqref="BB2:BB500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid browser_addon" promptTitle="browser_addon" prompt="Choose from the list" type="list">
-      <formula1>='_options'!$M$1:$M$4</formula1>
+      <formula1>browser_addon_options</formula1>
     </dataValidation>
     <dataValidation sqref="BE2:BE500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid advantage_plus_creative" promptTitle="advantage_plus_creative" prompt="Choose from the list" type="list">
-      <formula1>='_options'!$N$1:$N$2</formula1>
+      <formula1>advantage_plus_creative_options</formula1>
     </dataValidation>
     <dataValidation sqref="BF2:BF500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_add_overlays" promptTitle="adv_add_overlays" prompt="Choose from the list" type="list">
-      <formula1>='_options'!$O$1:$O$2</formula1>
+      <formula1>adv_add_overlays_options</formula1>
     </dataValidation>
     <dataValidation sqref="BG2:BG500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_image_touchups" promptTitle="adv_image_touchups" prompt="Choose from the list" type="list">
-      <formula1>='_options'!$P$1:$P$2</formula1>
+      <formula1>adv_image_touchups_options</formula1>
     </dataValidation>
     <dataValidation sqref="BH2:BH500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_music" promptTitle="adv_music" prompt="Choose from the list" type="list">
-      <formula1>='_options'!$Q$1:$Q$2</formula1>
+      <formula1>adv_music_options</formula1>
     </dataValidation>
     <dataValidation sqref="BI2:BI500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_text_generation" promptTitle="adv_text_generation" prompt="Choose from the list" type="list">
-      <formula1>='_options'!$R$1:$R$2</formula1>
+      <formula1>adv_text_generation_options</formula1>
     </dataValidation>
     <dataValidation sqref="BJ2:BJ500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_image_animation" promptTitle="adv_image_animation" prompt="Choose from the list" type="list">
-      <formula1>='_options'!$S$1:$S$2</formula1>
+      <formula1>adv_image_animation_options</formula1>
     </dataValidation>
     <dataValidation sqref="BK2:BK500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_product_tags" promptTitle="adv_product_tags" prompt="Choose from the list" type="list">
-      <formula1>='_options'!$T$1:$T$2</formula1>
+      <formula1>adv_product_tags_options</formula1>
     </dataValidation>
     <dataValidation sqref="BL2:BL500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_relevant_comments" promptTitle="adv_relevant_comments" prompt="Choose from the list" type="list">
-      <formula1>='_options'!$U$1:$U$2</formula1>
+      <formula1>adv_relevant_comments_options</formula1>
     </dataValidation>
     <dataValidation sqref="BM2:BM500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_enhance_cta" promptTitle="adv_enhance_cta" prompt="Choose from the list" type="list">
-      <formula1>='_options'!$V$1:$V$2</formula1>
+      <formula1>adv_enhance_cta_options</formula1>
     </dataValidation>
     <dataValidation sqref="BN2:BN500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_brightness_contrast" promptTitle="adv_brightness_contrast" prompt="Choose from the list" type="list">
-      <formula1>='_options'!$W$1:$W$2</formula1>
+      <formula1>adv_brightness_contrast_options</formula1>
     </dataValidation>
     <dataValidation sqref="BO2:BO500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_reveal_details" promptTitle="adv_reveal_details" prompt="Choose from the list" type="list">
-      <formula1>='_options'!$X$1:$X$2</formula1>
+      <formula1>adv_reveal_details_options</formula1>
     </dataValidation>
     <dataValidation sqref="BP2:BP500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_spotlights" promptTitle="adv_spotlights" prompt="Choose from the list" type="list">
-      <formula1>='_options'!$Y$1:$Y$2</formula1>
+      <formula1>adv_spotlights_options</formula1>
     </dataValidation>
     <dataValidation sqref="BQ2:BQ500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_text_overlay_translation" promptTitle="adv_text_overlay_translation" prompt="Choose from the list" type="list">
-      <formula1>='_options'!$Z$1:$Z$2</formula1>
+      <formula1>adv_text_overlay_translation_options</formula1>
     </dataValidation>
     <dataValidation sqref="BR2:BR500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_ig_video_subtitle" promptTitle="adv_ig_video_subtitle" prompt="Choose from the list" type="list">
-      <formula1>='_options'!$AA$1:$AA$2</formula1>
+      <formula1>adv_ig_video_subtitle_options</formula1>
     </dataValidation>
     <dataValidation sqref="BS2:BS500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_profile_card" promptTitle="adv_profile_card" prompt="Choose from the list" type="list">
-      <formula1>='_options'!$AB$1:$AB$2</formula1>
+      <formula1>adv_profile_card_options</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1107,681 +1132,823 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB21"/>
+  <dimension ref="A1:AB22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>OUTCOME_AWARENESS</t>
+          <t>campaign_objective</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>AUCTION</t>
+          <t>buying_type</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>special_ad_categories</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>LOWEST_COST_WITHOUT_CAP</t>
+          <t>campaign_bid_strategy</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>LOWEST_COST_WITHOUT_CAP</t>
+          <t>bid_strategy</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>standard</t>
+          <t>pacing_type</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>IMPRESSIONS</t>
+          <t>billing_event</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>REACH</t>
+          <t>optimization_goal</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>WEBSITE</t>
+          <t>destination_type</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>PURCHASE</t>
+          <t>custom_event_type</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>genders</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>SHOP_NOW</t>
+          <t>cta</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>browser_addon</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>advantage_plus_creative</t>
         </is>
       </c>
       <c r="O1" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>adv_add_overlays</t>
         </is>
       </c>
       <c r="P1" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>adv_image_touchups</t>
         </is>
       </c>
       <c r="Q1" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>adv_music</t>
         </is>
       </c>
       <c r="R1" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>adv_text_generation</t>
         </is>
       </c>
       <c r="S1" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>adv_image_animation</t>
         </is>
       </c>
       <c r="T1" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>adv_product_tags</t>
         </is>
       </c>
       <c r="U1" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>adv_relevant_comments</t>
         </is>
       </c>
       <c r="V1" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>adv_enhance_cta</t>
         </is>
       </c>
       <c r="W1" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>adv_brightness_contrast</t>
         </is>
       </c>
       <c r="X1" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>adv_reveal_details</t>
         </is>
       </c>
       <c r="Y1" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>adv_spotlights</t>
         </is>
       </c>
       <c r="Z1" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>adv_text_overlay_translation</t>
         </is>
       </c>
       <c r="AA1" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>adv_ig_video_subtitle</t>
         </is>
       </c>
       <c r="AB1" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>adv_profile_card</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>OUTCOME_TRAFFIC</t>
+          <t>OUTCOME_AWARENESS</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>RESERVED</t>
+          <t>AUCTION</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>HOUSING</t>
+          <t>NONE</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>LOWEST_COST_WITH_BID_CAP</t>
+          <t>LOWEST_COST_WITHOUT_CAP</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>LOWEST_COST_WITH_BID_CAP</t>
+          <t>LOWEST_COST_WITHOUT_CAP</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>no_pacing</t>
+          <t>standard</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>LINK_CLICKS</t>
+          <t>IMPRESSIONS</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>IMPRESSIONS</t>
+          <t>REACH</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>APP</t>
+          <t>WEBSITE</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>LEAD</t>
+          <t>PURCHASE</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>LEARN_MORE</t>
+          <t>SHOP_NOW</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>CALL</t>
+          <t>NONE</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>OUTCOME_ENGAGEMENT</t>
+          <t>OUTCOME_TRAFFIC</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>RESERVED</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>CREDIT</t>
+          <t>HOUSING</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>COST_CAP</t>
+          <t>LOWEST_COST_WITH_BID_CAP</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>COST_CAP</t>
+          <t>LOWEST_COST_WITH_BID_CAP</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>no_pacing</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>POST_ENGAGEMENT</t>
+          <t>LINK_CLICKS</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>LINK_CLICKS</t>
+          <t>IMPRESSIONS</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>MESSENGER</t>
+          <t>APP</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>COMPLETE_REGISTRATION</t>
+          <t>LEAD</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>1,2</t>
+          <t>2</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>SIGN_UP</t>
+          <t>LEARN_MORE</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>MESSENGER</t>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>OUTCOME_LEADS</t>
+          <t>OUTCOME_ENGAGEMENT</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>EMPLOYMENT</t>
+          <t>CREDIT</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>LOWEST_COST_WITH_MIN_ROAS</t>
+          <t>COST_CAP</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>LOWEST_COST_WITH_MIN_ROAS</t>
+          <t>COST_CAP</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>VIDEO_VIEWS</t>
+          <t>POST_ENGAGEMENT</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>LANDING_PAGE_VIEWS</t>
+          <t>LINK_CLICKS</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>INSTAGRAM_DIRECT</t>
+          <t>MESSENGER</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>ADD_TO_CART</t>
+          <t>COMPLETE_REGISTRATION</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>1,2</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>SUBSCRIBE</t>
+          <t>SIGN_UP</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>WHATSAPP</t>
+          <t>MESSENGER</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>OUTCOME_APP_PROMOTION</t>
+          <t>OUTCOME_LEADS</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ISSUES_ELECTIONS_POLITICS</t>
+          <t>EMPLOYMENT</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>LOWEST_COST_WITH_MIN_ROAS</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>LOWEST_COST_WITH_MIN_ROAS</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>THRUPLAY</t>
+          <t>VIDEO_VIEWS</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>POST_ENGAGEMENT</t>
+          <t>LANDING_PAGE_VIEWS</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
+          <t>INSTAGRAM_DIRECT</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>ADD_TO_CART</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>SUBSCRIBE</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
           <t>WHATSAPP</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>INITIATE_CHECKOUT</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>DOWNLOAD</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>OUTCOME_APP_PROMOTION</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>ISSUES_ELECTIONS_POLITICS</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>THRUPLAY</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>POST_ENGAGEMENT</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>WHATSAPP</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>INITIATE_CHECKOUT</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>DOWNLOAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
           <t>OUTCOME_SALES</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>ONLINE_GAMBLING_AND_GAMING</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>PAGE_LIKES</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>FACEBOOK</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>ADD_PAYMENT_INFO</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>BOOK_TRAVEL</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="C7" t="inlineStr">
+    <row r="8">
+      <c r="C8" t="inlineStr">
         <is>
           <t>FINANCIAL_PRODUCTS_SERVICES</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>VIDEO_VIEWS</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>ON_AD</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>VIEW_CONTENT</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>CONTACT_US</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>THRUPLAY</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>ON_POST</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>SEARCH</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>GET_OFFER</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="H9" t="inlineStr">
         <is>
-          <t>OFFSITE_CONVERSIONS</t>
+          <t>THRUPLAY</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>ON_PAGE</t>
+          <t>ON_POST</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>SUBSCRIBE</t>
+          <t>SEARCH</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>GET_QUOTE</t>
+          <t>GET_OFFER</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="H10" t="inlineStr">
         <is>
-          <t>VALUE</t>
+          <t>OFFSITE_CONVERSIONS</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>ON_EVENT</t>
+          <t>ON_PAGE</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>CONTACT</t>
+          <t>SUBSCRIBE</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>APPLY_NOW</t>
+          <t>GET_QUOTE</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="H11" t="inlineStr">
         <is>
-          <t>LEAD_GENERATION</t>
+          <t>VALUE</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>ON_VIDEO</t>
+          <t>ON_EVENT</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>DONATE</t>
+          <t>CONTACT</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>ORDER_NOW</t>
+          <t>APPLY_NOW</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="H12" t="inlineStr">
         <is>
-          <t>QUALITY_LEAD</t>
+          <t>LEAD_GENERATION</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>SHOP_AUTOMATIC</t>
+          <t>ON_VIDEO</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>OTHER</t>
+          <t>DONATE</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>DONATE_NOW</t>
+          <t>ORDER_NOW</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="H13" t="inlineStr">
         <is>
-          <t>CONVERSATIONS</t>
+          <t>QUALITY_LEAD</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>SHOP_AUTOMATIC</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>OTHER</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>INSTALL_APP</t>
+          <t>DONATE_NOW</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="H14" t="inlineStr">
         <is>
-          <t>APP_INSTALLS</t>
+          <t>CONVERSATIONS</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>USE_APP</t>
+          <t>INSTALL_APP</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="H15" t="inlineStr">
         <is>
+          <t>APP_INSTALLS</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>USE_APP</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="H16" t="inlineStr">
+        <is>
           <t>AD_RECALL_LIFT</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr">
+      <c r="L16" t="inlineStr">
         <is>
           <t>WATCH_MORE</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>LISTEN_NOW</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="L17" t="inlineStr">
         <is>
-          <t>SEND_MESSAGE</t>
+          <t>LISTEN_NOW</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="L18" t="inlineStr">
         <is>
-          <t>MESSAGE_PAGE</t>
+          <t>SEND_MESSAGE</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="L19" t="inlineStr">
         <is>
-          <t>GET_DIRECTIONS</t>
+          <t>MESSAGE_PAGE</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="L20" t="inlineStr">
         <is>
-          <t>CALL_NOW</t>
+          <t>GET_DIRECTIONS</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="L21" t="inlineStr">
+        <is>
+          <t>CALL_NOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="L22" t="inlineStr">
         <is>
           <t>NO_BUTTON</t>
         </is>

</xml_diff>

<commit_message>
existing-post / partnership: apply cta+link override and identity columns
- cta and link_url are no longer ignored when using existing_post_id
  or partnership_ad_code. They're set as a creative-level call_to
  _action that overrides the post's own CTA / destination URL on
  the rendered ad.
- partnership_ad_code now auto-sets branded_content_sharing_partner
  _id to the row's page_id (you, the sponsor). Two new optional
  columns override:
    branded_content_sponsor_page_id  -> which of your Pages is the
                                        sponsor (rare; defaults to
                                        page_id)
    branded_content_sponsor_ig_id    -> which of your IGs is shown
                                        as sponsor IG (defaults to
                                        instagram_user_id)
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BU2"/>
+  <dimension ref="A1:BW2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -491,8 +491,8 @@
     <col width="14" customWidth="1" min="43" max="43"/>
     <col width="18" customWidth="1" min="44" max="44"/>
     <col width="21" customWidth="1" min="45" max="45"/>
-    <col width="14" customWidth="1" min="46" max="46"/>
-    <col width="14" customWidth="1" min="47" max="47"/>
+    <col width="33" customWidth="1" min="46" max="46"/>
+    <col width="31" customWidth="1" min="47" max="47"/>
     <col width="14" customWidth="1" min="48" max="48"/>
     <col width="14" customWidth="1" min="49" max="49"/>
     <col width="14" customWidth="1" min="50" max="50"/>
@@ -501,24 +501,26 @@
     <col width="14" customWidth="1" min="53" max="53"/>
     <col width="14" customWidth="1" min="54" max="54"/>
     <col width="14" customWidth="1" min="55" max="55"/>
-    <col width="15" customWidth="1" min="56" max="56"/>
+    <col width="14" customWidth="1" min="56" max="56"/>
     <col width="14" customWidth="1" min="57" max="57"/>
-    <col width="19" customWidth="1" min="58" max="58"/>
-    <col width="25" customWidth="1" min="59" max="59"/>
-    <col width="18" customWidth="1" min="60" max="60"/>
-    <col width="20" customWidth="1" min="61" max="61"/>
-    <col width="14" customWidth="1" min="62" max="62"/>
-    <col width="21" customWidth="1" min="63" max="63"/>
-    <col width="21" customWidth="1" min="64" max="64"/>
-    <col width="18" customWidth="1" min="65" max="65"/>
-    <col width="23" customWidth="1" min="66" max="66"/>
-    <col width="17" customWidth="1" min="67" max="67"/>
-    <col width="25" customWidth="1" min="68" max="68"/>
-    <col width="20" customWidth="1" min="69" max="69"/>
-    <col width="16" customWidth="1" min="70" max="70"/>
-    <col width="30" customWidth="1" min="71" max="71"/>
-    <col width="23" customWidth="1" min="72" max="72"/>
-    <col width="18" customWidth="1" min="73" max="73"/>
+    <col width="15" customWidth="1" min="58" max="58"/>
+    <col width="14" customWidth="1" min="59" max="59"/>
+    <col width="19" customWidth="1" min="60" max="60"/>
+    <col width="25" customWidth="1" min="61" max="61"/>
+    <col width="18" customWidth="1" min="62" max="62"/>
+    <col width="20" customWidth="1" min="63" max="63"/>
+    <col width="14" customWidth="1" min="64" max="64"/>
+    <col width="21" customWidth="1" min="65" max="65"/>
+    <col width="21" customWidth="1" min="66" max="66"/>
+    <col width="18" customWidth="1" min="67" max="67"/>
+    <col width="23" customWidth="1" min="68" max="68"/>
+    <col width="17" customWidth="1" min="69" max="69"/>
+    <col width="25" customWidth="1" min="70" max="70"/>
+    <col width="20" customWidth="1" min="71" max="71"/>
+    <col width="16" customWidth="1" min="72" max="72"/>
+    <col width="30" customWidth="1" min="73" max="73"/>
+    <col width="23" customWidth="1" min="74" max="74"/>
+    <col width="18" customWidth="1" min="75" max="75"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -749,140 +751,150 @@
       </c>
       <c r="AT1" t="inlineStr">
         <is>
+          <t>branded_content_sponsor_page_id</t>
+        </is>
+      </c>
+      <c r="AU1" t="inlineStr">
+        <is>
+          <t>branded_content_sponsor_ig_id</t>
+        </is>
+      </c>
+      <c r="AV1" t="inlineStr">
+        <is>
           <t>image_url</t>
         </is>
       </c>
-      <c r="AU1" t="inlineStr">
+      <c r="AW1" t="inlineStr">
         <is>
           <t>video_id</t>
         </is>
       </c>
-      <c r="AV1" t="inlineStr">
+      <c r="AX1" t="inlineStr">
         <is>
           <t>video_url</t>
         </is>
       </c>
-      <c r="AW1" t="inlineStr">
+      <c r="AY1" t="inlineStr">
         <is>
           <t>primary_text</t>
         </is>
       </c>
-      <c r="AX1" t="inlineStr">
+      <c r="AZ1" t="inlineStr">
         <is>
           <t>headline</t>
         </is>
       </c>
-      <c r="AY1" t="inlineStr">
+      <c r="BA1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="AZ1" t="inlineStr">
+      <c r="BB1" t="inlineStr">
         <is>
           <t>link_url</t>
         </is>
       </c>
-      <c r="BA1" t="inlineStr">
+      <c r="BC1" t="inlineStr">
         <is>
           <t>display_link</t>
         </is>
       </c>
-      <c r="BB1" t="inlineStr">
+      <c r="BD1" t="inlineStr">
         <is>
           <t>url_tags</t>
         </is>
       </c>
-      <c r="BC1" t="inlineStr">
+      <c r="BE1" t="inlineStr">
         <is>
           <t>cta</t>
         </is>
       </c>
-      <c r="BD1" t="inlineStr">
+      <c r="BF1" t="inlineStr">
         <is>
           <t>browser_addon</t>
         </is>
       </c>
-      <c r="BE1" t="inlineStr">
+      <c r="BG1" t="inlineStr">
         <is>
           <t>phone_number</t>
         </is>
       </c>
-      <c r="BF1" t="inlineStr">
+      <c r="BH1" t="inlineStr">
         <is>
           <t>conversion_domain</t>
         </is>
       </c>
-      <c r="BG1" t="inlineStr">
+      <c r="BI1" t="inlineStr">
         <is>
           <t>advantage_plus_creative</t>
         </is>
       </c>
-      <c r="BH1" t="inlineStr">
+      <c r="BJ1" t="inlineStr">
         <is>
           <t>adv_add_overlays</t>
         </is>
       </c>
-      <c r="BI1" t="inlineStr">
+      <c r="BK1" t="inlineStr">
         <is>
           <t>adv_image_touchups</t>
         </is>
       </c>
-      <c r="BJ1" t="inlineStr">
+      <c r="BL1" t="inlineStr">
         <is>
           <t>adv_music</t>
         </is>
       </c>
-      <c r="BK1" t="inlineStr">
+      <c r="BM1" t="inlineStr">
         <is>
           <t>adv_text_generation</t>
         </is>
       </c>
-      <c r="BL1" t="inlineStr">
+      <c r="BN1" t="inlineStr">
         <is>
           <t>adv_image_animation</t>
         </is>
       </c>
-      <c r="BM1" t="inlineStr">
+      <c r="BO1" t="inlineStr">
         <is>
           <t>adv_product_tags</t>
         </is>
       </c>
-      <c r="BN1" t="inlineStr">
+      <c r="BP1" t="inlineStr">
         <is>
           <t>adv_relevant_comments</t>
         </is>
       </c>
-      <c r="BO1" t="inlineStr">
+      <c r="BQ1" t="inlineStr">
         <is>
           <t>adv_enhance_cta</t>
         </is>
       </c>
-      <c r="BP1" t="inlineStr">
+      <c r="BR1" t="inlineStr">
         <is>
           <t>adv_brightness_contrast</t>
         </is>
       </c>
-      <c r="BQ1" t="inlineStr">
+      <c r="BS1" t="inlineStr">
         <is>
           <t>adv_reveal_details</t>
         </is>
       </c>
-      <c r="BR1" t="inlineStr">
+      <c r="BT1" t="inlineStr">
         <is>
           <t>adv_spotlights</t>
         </is>
       </c>
-      <c r="BS1" t="inlineStr">
+      <c r="BU1" t="inlineStr">
         <is>
           <t>adv_text_overlay_translation</t>
         </is>
       </c>
-      <c r="BT1" t="inlineStr">
+      <c r="BV1" t="inlineStr">
         <is>
           <t>adv_ig_video_subtitle</t>
         </is>
       </c>
-      <c r="BU1" t="inlineStr">
+      <c r="BW1" t="inlineStr">
         <is>
           <t>adv_profile_card</t>
         </is>
@@ -988,53 +1000,53 @@
       </c>
       <c r="AR2" t="inlineStr"/>
       <c r="AS2" t="inlineStr"/>
-      <c r="AT2" t="inlineStr">
+      <c r="AT2" t="inlineStr"/>
+      <c r="AU2" t="inlineStr"/>
+      <c r="AV2" t="inlineStr">
         <is>
           <t>https://example.com/image.jpg</t>
         </is>
       </c>
-      <c r="AU2" t="inlineStr"/>
-      <c r="AV2" t="inlineStr"/>
-      <c r="AW2" t="inlineStr">
+      <c r="AW2" t="inlineStr"/>
+      <c r="AX2" t="inlineStr"/>
+      <c r="AY2" t="inlineStr">
         <is>
           <t>Body copy goes here.</t>
         </is>
       </c>
-      <c r="AX2" t="inlineStr">
+      <c r="AZ2" t="inlineStr">
         <is>
           <t>Your headline</t>
         </is>
       </c>
-      <c r="AY2" t="inlineStr">
+      <c r="BA2" t="inlineStr">
         <is>
           <t>Short description.</t>
         </is>
       </c>
-      <c r="AZ2" t="inlineStr">
+      <c r="BB2" t="inlineStr">
         <is>
           <t>https://example.com/landing</t>
         </is>
       </c>
-      <c r="BA2" t="inlineStr">
+      <c r="BC2" t="inlineStr">
         <is>
           <t>example.com</t>
         </is>
       </c>
-      <c r="BB2" t="inlineStr"/>
-      <c r="BC2" t="inlineStr">
+      <c r="BD2" t="inlineStr"/>
+      <c r="BE2" t="inlineStr">
         <is>
           <t>SHOP_NOW</t>
         </is>
       </c>
-      <c r="BD2" t="inlineStr"/>
-      <c r="BE2" t="inlineStr"/>
-      <c r="BF2" t="inlineStr">
+      <c r="BF2" t="inlineStr"/>
+      <c r="BG2" t="inlineStr"/>
+      <c r="BH2" t="inlineStr">
         <is>
           <t>example.com</t>
         </is>
       </c>
-      <c r="BG2" t="inlineStr"/>
-      <c r="BH2" t="inlineStr"/>
       <c r="BI2" t="inlineStr"/>
       <c r="BJ2" t="inlineStr"/>
       <c r="BK2" t="inlineStr"/>
@@ -1048,6 +1060,8 @@
       <c r="BS2" t="inlineStr"/>
       <c r="BT2" t="inlineStr"/>
       <c r="BU2" t="inlineStr"/>
+      <c r="BV2" t="inlineStr"/>
+      <c r="BW2" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="28">
@@ -1084,55 +1098,55 @@
     <dataValidation sqref="AK2:AK500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid genders" promptTitle="genders" prompt="Choose from the list" type="list">
       <formula1>genders_options</formula1>
     </dataValidation>
-    <dataValidation sqref="BC2:BC500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid cta" promptTitle="cta" prompt="Choose from the list" type="list">
+    <dataValidation sqref="BE2:BE500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid cta" promptTitle="cta" prompt="Choose from the list" type="list">
       <formula1>cta_options</formula1>
     </dataValidation>
-    <dataValidation sqref="BD2:BD500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid browser_addon" promptTitle="browser_addon" prompt="Choose from the list" type="list">
+    <dataValidation sqref="BF2:BF500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid browser_addon" promptTitle="browser_addon" prompt="Choose from the list" type="list">
       <formula1>browser_addon_options</formula1>
     </dataValidation>
-    <dataValidation sqref="BG2:BG500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid advantage_plus_creative" promptTitle="advantage_plus_creative" prompt="Choose from the list" type="list">
+    <dataValidation sqref="BI2:BI500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid advantage_plus_creative" promptTitle="advantage_plus_creative" prompt="Choose from the list" type="list">
       <formula1>advantage_plus_creative_options</formula1>
     </dataValidation>
-    <dataValidation sqref="BH2:BH500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_add_overlays" promptTitle="adv_add_overlays" prompt="Choose from the list" type="list">
+    <dataValidation sqref="BJ2:BJ500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_add_overlays" promptTitle="adv_add_overlays" prompt="Choose from the list" type="list">
       <formula1>adv_add_overlays_options</formula1>
     </dataValidation>
-    <dataValidation sqref="BI2:BI500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_image_touchups" promptTitle="adv_image_touchups" prompt="Choose from the list" type="list">
+    <dataValidation sqref="BK2:BK500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_image_touchups" promptTitle="adv_image_touchups" prompt="Choose from the list" type="list">
       <formula1>adv_image_touchups_options</formula1>
     </dataValidation>
-    <dataValidation sqref="BJ2:BJ500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_music" promptTitle="adv_music" prompt="Choose from the list" type="list">
+    <dataValidation sqref="BL2:BL500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_music" promptTitle="adv_music" prompt="Choose from the list" type="list">
       <formula1>adv_music_options</formula1>
     </dataValidation>
-    <dataValidation sqref="BK2:BK500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_text_generation" promptTitle="adv_text_generation" prompt="Choose from the list" type="list">
+    <dataValidation sqref="BM2:BM500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_text_generation" promptTitle="adv_text_generation" prompt="Choose from the list" type="list">
       <formula1>adv_text_generation_options</formula1>
     </dataValidation>
-    <dataValidation sqref="BL2:BL500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_image_animation" promptTitle="adv_image_animation" prompt="Choose from the list" type="list">
+    <dataValidation sqref="BN2:BN500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_image_animation" promptTitle="adv_image_animation" prompt="Choose from the list" type="list">
       <formula1>adv_image_animation_options</formula1>
     </dataValidation>
-    <dataValidation sqref="BM2:BM500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_product_tags" promptTitle="adv_product_tags" prompt="Choose from the list" type="list">
+    <dataValidation sqref="BO2:BO500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_product_tags" promptTitle="adv_product_tags" prompt="Choose from the list" type="list">
       <formula1>adv_product_tags_options</formula1>
     </dataValidation>
-    <dataValidation sqref="BN2:BN500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_relevant_comments" promptTitle="adv_relevant_comments" prompt="Choose from the list" type="list">
+    <dataValidation sqref="BP2:BP500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_relevant_comments" promptTitle="adv_relevant_comments" prompt="Choose from the list" type="list">
       <formula1>adv_relevant_comments_options</formula1>
     </dataValidation>
-    <dataValidation sqref="BO2:BO500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_enhance_cta" promptTitle="adv_enhance_cta" prompt="Choose from the list" type="list">
+    <dataValidation sqref="BQ2:BQ500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_enhance_cta" promptTitle="adv_enhance_cta" prompt="Choose from the list" type="list">
       <formula1>adv_enhance_cta_options</formula1>
     </dataValidation>
-    <dataValidation sqref="BP2:BP500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_brightness_contrast" promptTitle="adv_brightness_contrast" prompt="Choose from the list" type="list">
+    <dataValidation sqref="BR2:BR500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_brightness_contrast" promptTitle="adv_brightness_contrast" prompt="Choose from the list" type="list">
       <formula1>adv_brightness_contrast_options</formula1>
     </dataValidation>
-    <dataValidation sqref="BQ2:BQ500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_reveal_details" promptTitle="adv_reveal_details" prompt="Choose from the list" type="list">
+    <dataValidation sqref="BS2:BS500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_reveal_details" promptTitle="adv_reveal_details" prompt="Choose from the list" type="list">
       <formula1>adv_reveal_details_options</formula1>
     </dataValidation>
-    <dataValidation sqref="BR2:BR500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_spotlights" promptTitle="adv_spotlights" prompt="Choose from the list" type="list">
+    <dataValidation sqref="BT2:BT500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_spotlights" promptTitle="adv_spotlights" prompt="Choose from the list" type="list">
       <formula1>adv_spotlights_options</formula1>
     </dataValidation>
-    <dataValidation sqref="BS2:BS500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_text_overlay_translation" promptTitle="adv_text_overlay_translation" prompt="Choose from the list" type="list">
+    <dataValidation sqref="BU2:BU500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_text_overlay_translation" promptTitle="adv_text_overlay_translation" prompt="Choose from the list" type="list">
       <formula1>adv_text_overlay_translation_options</formula1>
     </dataValidation>
-    <dataValidation sqref="BT2:BT500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_ig_video_subtitle" promptTitle="adv_ig_video_subtitle" prompt="Choose from the list" type="list">
+    <dataValidation sqref="BV2:BV500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_ig_video_subtitle" promptTitle="adv_ig_video_subtitle" prompt="Choose from the list" type="list">
       <formula1>adv_ig_video_subtitle_options</formula1>
     </dataValidation>
-    <dataValidation sqref="BU2:BU500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_profile_card" promptTitle="adv_profile_card" prompt="Choose from the list" type="list">
+    <dataValidation sqref="BW2:BW500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_profile_card" promptTitle="adv_profile_card" prompt="Choose from the list" type="list">
       <formula1>adv_profile_card_options</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>